<commit_message>
Update FWI forecast and geographic report
</commit_message>
<xml_diff>
--- a/data/FARS_FWI_GeoReport.xlsx
+++ b/data/FARS_FWI_GeoReport.xlsx
@@ -46,6 +46,24 @@
     <t>طبقه خطر</t>
   </si>
   <si>
+    <t>منطقه شکار ممنوع بصيران</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع دره باغ</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع شیکوه</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه دراء</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده ارژن و پريشان</t>
+  </si>
+  <si>
+    <t>پناهگاه حيات وحش دره باغ</t>
+  </si>
+  <si>
     <t>منطقه حفاظت شده بهرام گور</t>
   </si>
   <si>
@@ -55,112 +73,94 @@
     <t>منطقه شکار ممنوع کوهستان</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع کوه دراء</t>
+    <t>منطقه شکار ممنوع مزايجان</t>
   </si>
   <si>
     <t>منطقه شکار ممنوع مل بلند</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع شیکوه</t>
+    <t>منطقه شکار ممنوع توت سياه</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع بناب</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده هرمود</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع دالان</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده میانجنگل فسا</t>
+  </si>
+  <si>
+    <t>پارک ملي بختگان</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع پادنا</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه هوا و</t>
   </si>
   <si>
     <t>منطقه شکار ممنوع مهارلو</t>
   </si>
   <si>
+    <t>پناهگاه حيات وحش بختگان</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده برم فیروز</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه گورم</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه سياه</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده تنگ بستانک</t>
+  </si>
+  <si>
     <t>پارک ملی بمو</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع توت سياه</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده میانجنگل فسا</t>
+    <t>منطقه شکار ممن.ع آق جلو</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه خرسي</t>
   </si>
   <si>
     <t>منطقه شکار ممنوع روشن کوه</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع دره باغ</t>
+    <t>منطقه حفاظت شده ماله گاله</t>
   </si>
   <si>
     <t>منطقه حفاظت شده تنگ سرخ و کوه قلات</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع بصيران</t>
-  </si>
-  <si>
-    <t>پناهگاه حيات وحش بختگان</t>
-  </si>
-  <si>
-    <t>پناهگاه حيات وحش دره باغ</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممن.ع آق جلو</t>
-  </si>
-  <si>
-    <t>پارک ملي بختگان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع مزايجان</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده تنگ بستانک</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده برم فیروز</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده ماله گاله</t>
-  </si>
-  <si>
     <t>منطقه شکار ممنوع خرمنکوه</t>
   </si>
   <si>
     <t>منطقه شکار ممنوع کوه خم</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع کوه گورم</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده ارژن و پريشان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع بناب</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوه سياه</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوه خرسي</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع دالان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوه هوا و</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع پادنا</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده هرمود</t>
-  </si>
-  <si>
     <t>منطقه شکار ممنوع چاه نفت</t>
   </si>
   <si>
     <t>منطقه حفاظت شده مارگون</t>
   </si>
   <si>
+    <t>مناطق حفاظت‌شده</t>
+  </si>
+  <si>
     <t>مناطق ممنوعه شکار</t>
   </si>
   <si>
-    <t>مناطق حفاظت‌شده</t>
-  </si>
-  <si>
-    <t>1405-06-01</t>
-  </si>
-  <si>
-    <t>2026-08-23</t>
+    <t>1405-06-02</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
   </si>
   <si>
     <t>بسیار شدید</t>
@@ -628,16 +628,16 @@
         <v>47</v>
       </c>
       <c r="E2">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F2">
-        <v>81.52</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G2">
-        <v>85.23999999999999</v>
+        <v>80.36</v>
       </c>
       <c r="H2">
-        <v>89.76000000000001</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="I2" t="s">
         <v>48</v>
@@ -657,16 +657,16 @@
         <v>47</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F3">
-        <v>81.52</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="G3">
-        <v>81.52</v>
+        <v>79.47</v>
       </c>
       <c r="H3">
-        <v>81.52</v>
+        <v>84.61</v>
       </c>
       <c r="I3" t="s">
         <v>48</v>
@@ -677,7 +677,7 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
         <v>46</v>
@@ -686,16 +686,16 @@
         <v>47</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4">
-        <v>80.7</v>
+        <v>76.53</v>
       </c>
       <c r="G4">
-        <v>80.7</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="H4">
-        <v>80.7</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="I4" t="s">
         <v>48</v>
@@ -706,7 +706,7 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
         <v>46</v>
@@ -718,13 +718,13 @@
         <v>33</v>
       </c>
       <c r="F5">
-        <v>68.67</v>
+        <v>66.78</v>
       </c>
       <c r="G5">
-        <v>78.05</v>
+        <v>77.58</v>
       </c>
       <c r="H5">
-        <v>88.08</v>
+        <v>88.05</v>
       </c>
       <c r="I5" t="s">
         <v>48</v>
@@ -744,16 +744,16 @@
         <v>47</v>
       </c>
       <c r="E6">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="F6">
-        <v>74.81</v>
+        <v>53.58</v>
       </c>
       <c r="G6">
-        <v>77.33</v>
+        <v>77.37</v>
       </c>
       <c r="H6">
-        <v>80.91</v>
+        <v>89.31999999999999</v>
       </c>
       <c r="I6" t="s">
         <v>48</v>
@@ -776,13 +776,13 @@
         <v>3</v>
       </c>
       <c r="F7">
-        <v>73.73</v>
+        <v>74.11</v>
       </c>
       <c r="G7">
-        <v>75.52</v>
+        <v>77.26000000000001</v>
       </c>
       <c r="H7">
-        <v>77.01000000000001</v>
+        <v>80.8</v>
       </c>
       <c r="I7" t="s">
         <v>48</v>
@@ -802,16 +802,16 @@
         <v>47</v>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F8">
-        <v>67.23999999999999</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="G8">
-        <v>73.73</v>
+        <v>77.12</v>
       </c>
       <c r="H8">
-        <v>76.23999999999999</v>
+        <v>86.15000000000001</v>
       </c>
       <c r="I8" t="s">
         <v>48</v>
@@ -822,7 +822,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
         <v>46</v>
@@ -831,16 +831,16 @@
         <v>47</v>
       </c>
       <c r="E9">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F9">
-        <v>63.69</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="G9">
-        <v>72.41</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="H9">
-        <v>78.45</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="I9" t="s">
         <v>48</v>
@@ -851,7 +851,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
         <v>46</v>
@@ -860,16 +860,16 @@
         <v>47</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>70.17</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="G10">
-        <v>72.15000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="H10">
-        <v>74.83</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="I10" t="s">
         <v>48</v>
@@ -889,16 +889,16 @@
         <v>47</v>
       </c>
       <c r="E11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F11">
-        <v>68.38</v>
+        <v>56.57</v>
       </c>
       <c r="G11">
-        <v>71.70999999999999</v>
+        <v>70.98999999999999</v>
       </c>
       <c r="H11">
-        <v>76.62</v>
+        <v>77.11</v>
       </c>
       <c r="I11" t="s">
         <v>48</v>
@@ -909,7 +909,7 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>46</v>
@@ -918,19 +918,19 @@
         <v>47</v>
       </c>
       <c r="E12">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F12">
-        <v>65.36</v>
+        <v>65.37</v>
       </c>
       <c r="G12">
-        <v>70.86</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="H12">
-        <v>78.40000000000001</v>
+        <v>72.02</v>
       </c>
       <c r="I12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -938,7 +938,7 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
         <v>46</v>
@@ -947,19 +947,19 @@
         <v>47</v>
       </c>
       <c r="E13">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F13">
-        <v>69.03</v>
+        <v>66.33</v>
       </c>
       <c r="G13">
-        <v>70.39</v>
+        <v>68.72</v>
       </c>
       <c r="H13">
-        <v>73.86</v>
+        <v>70.25</v>
       </c>
       <c r="I13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -976,19 +976,19 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="F14">
-        <v>69.26000000000001</v>
+        <v>57.42</v>
       </c>
       <c r="G14">
-        <v>70.39</v>
+        <v>68.53</v>
       </c>
       <c r="H14">
-        <v>71.87</v>
+        <v>78.69</v>
       </c>
       <c r="I14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1005,19 +1005,19 @@
         <v>47</v>
       </c>
       <c r="E15">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F15">
-        <v>62.08</v>
+        <v>57.03</v>
       </c>
       <c r="G15">
-        <v>70.15000000000001</v>
+        <v>68.45</v>
       </c>
       <c r="H15">
-        <v>77.11</v>
+        <v>79.31</v>
       </c>
       <c r="I15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1034,16 +1034,16 @@
         <v>47</v>
       </c>
       <c r="E16">
-        <v>117</v>
+        <v>8</v>
       </c>
       <c r="F16">
-        <v>57.16</v>
+        <v>64.98</v>
       </c>
       <c r="G16">
-        <v>69.67</v>
+        <v>67.3</v>
       </c>
       <c r="H16">
-        <v>91.62</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="I16" t="s">
         <v>49</v>
@@ -1054,7 +1054,7 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
         <v>46</v>
@@ -1063,16 +1063,16 @@
         <v>47</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="F17">
-        <v>69.03</v>
+        <v>61.35</v>
       </c>
       <c r="G17">
-        <v>69.43000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="H17">
-        <v>69.66</v>
+        <v>68</v>
       </c>
       <c r="I17" t="s">
         <v>49</v>
@@ -1092,16 +1092,16 @@
         <v>47</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>65</v>
       </c>
       <c r="F18">
-        <v>68</v>
+        <v>53.87</v>
       </c>
       <c r="G18">
-        <v>68.81</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="H18">
-        <v>69.62</v>
+        <v>79.04000000000001</v>
       </c>
       <c r="I18" t="s">
         <v>49</v>
@@ -1121,16 +1121,16 @@
         <v>47</v>
       </c>
       <c r="E19">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="F19">
-        <v>57.16</v>
+        <v>57.43</v>
       </c>
       <c r="G19">
-        <v>68.73999999999999</v>
+        <v>64.97</v>
       </c>
       <c r="H19">
-        <v>91.62</v>
+        <v>71.63</v>
       </c>
       <c r="I19" t="s">
         <v>49</v>
@@ -1141,7 +1141,7 @@
         <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C20" t="s">
         <v>46</v>
@@ -1150,16 +1150,16 @@
         <v>47</v>
       </c>
       <c r="E20">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="F20">
-        <v>54.82</v>
+        <v>58.41</v>
       </c>
       <c r="G20">
-        <v>68.37</v>
+        <v>64.81</v>
       </c>
       <c r="H20">
-        <v>77.16</v>
+        <v>75.31</v>
       </c>
       <c r="I20" t="s">
         <v>49</v>
@@ -1179,16 +1179,16 @@
         <v>47</v>
       </c>
       <c r="E21">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F21">
-        <v>66.72</v>
+        <v>58.95</v>
       </c>
       <c r="G21">
-        <v>68.11</v>
+        <v>64.56</v>
       </c>
       <c r="H21">
-        <v>70.06</v>
+        <v>68.47</v>
       </c>
       <c r="I21" t="s">
         <v>49</v>
@@ -1199,7 +1199,7 @@
         <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C22" t="s">
         <v>46</v>
@@ -1208,16 +1208,16 @@
         <v>47</v>
       </c>
       <c r="E22">
-        <v>8</v>
+        <v>117</v>
       </c>
       <c r="F22">
-        <v>65.19</v>
+        <v>53.87</v>
       </c>
       <c r="G22">
-        <v>67.34</v>
+        <v>64.41</v>
       </c>
       <c r="H22">
-        <v>69.11</v>
+        <v>79.04000000000001</v>
       </c>
       <c r="I22" t="s">
         <v>49</v>
@@ -1228,7 +1228,7 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C23" t="s">
         <v>46</v>
@@ -1237,16 +1237,16 @@
         <v>47</v>
       </c>
       <c r="E23">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F23">
-        <v>60.4</v>
+        <v>63.45</v>
       </c>
       <c r="G23">
-        <v>66.06</v>
+        <v>64.12</v>
       </c>
       <c r="H23">
-        <v>69.47</v>
+        <v>65.66</v>
       </c>
       <c r="I23" t="s">
         <v>49</v>
@@ -1257,7 +1257,7 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
         <v>46</v>
@@ -1266,16 +1266,16 @@
         <v>47</v>
       </c>
       <c r="E24">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F24">
-        <v>61.82</v>
+        <v>59.17</v>
       </c>
       <c r="G24">
-        <v>65.43000000000001</v>
+        <v>64.11</v>
       </c>
       <c r="H24">
-        <v>70.59</v>
+        <v>71.27</v>
       </c>
       <c r="I24" t="s">
         <v>49</v>
@@ -1286,7 +1286,7 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25" t="s">
         <v>46</v>
@@ -1295,16 +1295,16 @@
         <v>47</v>
       </c>
       <c r="E25">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F25">
-        <v>60.36</v>
+        <v>56.09</v>
       </c>
       <c r="G25">
-        <v>65.28</v>
+        <v>63.92</v>
       </c>
       <c r="H25">
-        <v>70.51000000000001</v>
+        <v>68.08</v>
       </c>
       <c r="I25" t="s">
         <v>49</v>
@@ -1324,16 +1324,16 @@
         <v>47</v>
       </c>
       <c r="E26">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="F26">
-        <v>61.56</v>
+        <v>60.74</v>
       </c>
       <c r="G26">
-        <v>65.14</v>
+        <v>63.92</v>
       </c>
       <c r="H26">
-        <v>69.06</v>
+        <v>66.68000000000001</v>
       </c>
       <c r="I26" t="s">
         <v>49</v>
@@ -1344,7 +1344,7 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
         <v>46</v>
@@ -1353,16 +1353,16 @@
         <v>47</v>
       </c>
       <c r="E27">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F27">
-        <v>53.26</v>
+        <v>58.31</v>
       </c>
       <c r="G27">
-        <v>64.61</v>
+        <v>63.77</v>
       </c>
       <c r="H27">
-        <v>79.86</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="I27" t="s">
         <v>49</v>
@@ -1373,7 +1373,7 @@
         <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C28" t="s">
         <v>46</v>
@@ -1382,16 +1382,16 @@
         <v>47</v>
       </c>
       <c r="E28">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F28">
-        <v>54.45</v>
+        <v>61.51</v>
       </c>
       <c r="G28">
-        <v>64.42</v>
+        <v>62.04</v>
       </c>
       <c r="H28">
-        <v>77.54000000000001</v>
+        <v>62.58</v>
       </c>
       <c r="I28" t="s">
         <v>49</v>
@@ -1402,7 +1402,7 @@
         <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C29" t="s">
         <v>46</v>
@@ -1411,16 +1411,16 @@
         <v>47</v>
       </c>
       <c r="E29">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="F29">
-        <v>60.82</v>
+        <v>50.8</v>
       </c>
       <c r="G29">
-        <v>64.09</v>
+        <v>61.83</v>
       </c>
       <c r="H29">
-        <v>67.48</v>
+        <v>75.52</v>
       </c>
       <c r="I29" t="s">
         <v>49</v>
@@ -1431,7 +1431,7 @@
         <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C30" t="s">
         <v>46</v>
@@ -1440,16 +1440,16 @@
         <v>47</v>
       </c>
       <c r="E30">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="F30">
-        <v>55.45</v>
+        <v>54.29</v>
       </c>
       <c r="G30">
-        <v>63.4</v>
+        <v>60.67</v>
       </c>
       <c r="H30">
-        <v>77.14</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="I30" t="s">
         <v>49</v>
@@ -1469,16 +1469,16 @@
         <v>47</v>
       </c>
       <c r="E31">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F31">
-        <v>57.87</v>
+        <v>55.64</v>
       </c>
       <c r="G31">
-        <v>62.32</v>
+        <v>59.9</v>
       </c>
       <c r="H31">
-        <v>73.55</v>
+        <v>64.58</v>
       </c>
       <c r="I31" t="s">
         <v>49</v>
@@ -1498,16 +1498,16 @@
         <v>47</v>
       </c>
       <c r="E32">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="F32">
-        <v>55.91</v>
+        <v>58.69</v>
       </c>
       <c r="G32">
-        <v>61.06</v>
+        <v>59.83</v>
       </c>
       <c r="H32">
-        <v>71.29000000000001</v>
+        <v>61.73</v>
       </c>
       <c r="I32" t="s">
         <v>49</v>
@@ -1518,7 +1518,7 @@
         <v>40</v>
       </c>
       <c r="B33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C33" t="s">
         <v>46</v>
@@ -1527,16 +1527,16 @@
         <v>47</v>
       </c>
       <c r="E33">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F33">
-        <v>54.13</v>
+        <v>57.7</v>
       </c>
       <c r="G33">
-        <v>60.14</v>
+        <v>59.64</v>
       </c>
       <c r="H33">
-        <v>71.3</v>
+        <v>63.59</v>
       </c>
       <c r="I33" t="s">
         <v>49</v>
@@ -1556,16 +1556,16 @@
         <v>47</v>
       </c>
       <c r="E34">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F34">
-        <v>49.37</v>
+        <v>53.67</v>
       </c>
       <c r="G34">
-        <v>55.64</v>
+        <v>57.25</v>
       </c>
       <c r="H34">
-        <v>63.2</v>
+        <v>61.02</v>
       </c>
       <c r="I34" t="s">
         <v>49</v>
@@ -1576,7 +1576,7 @@
         <v>42</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C35" t="s">
         <v>46</v>
@@ -1596,7 +1596,7 @@
         <v>43</v>
       </c>
       <c r="B36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C36" t="s">
         <v>46</v>

</xml_diff>